<commit_message>
feat: onboard Bhikshu Tattoo Studio with custom zen ink palette, AI review drafts and printable QR stand
</commit_message>
<xml_diff>
--- a/TrueReview_Business_Registry.xlsx
+++ b/TrueReview_Business_Registry.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -613,9 +613,80 @@
         <v>/qr/example-dental</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Bhikshu Tattoo Studio</v>
+      </c>
+      <c r="B4" t="str">
+        <v>bhikshu-tattoo</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Tattoo &amp; Body Art Studio</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Viman Nagar, Pune • Connecting Stories to Tattoo</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Connecting your stories to your tattoo with peace &amp; precision. Share your ink journey on Google.</v>
+      </c>
+      <c r="F4" t="str">
+        <v>https://www.google.com/maps/place/Bhikshu+Tattoo+Studio+%7C+Best+tattoo+studio+in+pune/@18.5654478,73.9105924,112m/data=!3m1!1e3!4m8!3m7!1s0x3bc2c15ecc1b8797:0x315b9b1fa5949c21!8m2!3d18.5654477!4d73.9109004!9m1!1b1!16s%2Fg%2F11qnttbv42?entry=ttu&amp;g_ep=EgoyMDI2MTAyMC4wIKXMDSoASAFQAw%3D%3D</v>
+      </c>
+      <c r="G4" t="str">
+        <v>https://maps.app.goo.gl/ZWi4gTXhM4aZ4pS79</v>
+      </c>
+      <c r="H4" t="str">
+        <v>+91 96899 76453</v>
+      </c>
+      <c r="I4" t="str">
+        <v>919689976453</v>
+      </c>
+      <c r="J4" t="str">
+        <v>https://www.bhikshutattoostudio.com/</v>
+      </c>
+      <c r="K4" t="str">
+        <v>@bhikshu_tattoo</v>
+      </c>
+      <c r="L4" t="str">
+        <v>@bhikshutattoo</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Lane No.12, Row House 3, Konark Nagar, CCD Chowk, opp. Udaan Bio-Diversity Park, Viman Nagar, Pune, Maharashtra 411014</v>
+      </c>
+      <c r="N4">
+        <v>5</v>
+      </c>
+      <c r="O4">
+        <v>403</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Custom Tattoo Design; Realism &amp; Portraits; Mandala &amp; Fine Line; Tribal &amp; Maori; Black &amp; Grey; Script &amp; Lettering; Sculpture Tattoo; Body Piercing</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>100% Sterile &amp; Hygiene First; Incredibly Fine Lines; Peaceful Studio Ambience; Patient &amp; Gentle Artists; Meaningful Custom Design; Clear Aftercare Guidance; Transparent Pricing</v>
+      </c>
+      <c r="R4" t="str">
+        <v>/assets/bhikshu-logo.png</v>
+      </c>
+      <c r="S4" t="str">
+        <v>#4A554D</v>
+      </c>
+      <c r="T4" t="str">
+        <v>#FAF9F5</v>
+      </c>
+      <c r="U4" t="str">
+        <v>Active</v>
+      </c>
+      <c r="V4" t="str">
+        <v>/r/bhikshu-tattoo</v>
+      </c>
+      <c r="W4" t="str">
+        <v>/qr/bhikshu-tattoo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(bhikshu): add POWERED BY @phoenixtech.co badge in top-right corner with Sora font
</commit_message>
<xml_diff>
--- a/TrueReview_Business_Registry.xlsx
+++ b/TrueReview_Business_Registry.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -684,9 +684,80 @@
         <v>/qr/bhikshu-tattoo</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Naad Jamroom &amp; Studio</v>
+      </c>
+      <c r="B5" t="str">
+        <v>naadjamroom</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Jam Room &amp; Audio Recording Studio</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Kharadi, Pune • Jam Room &amp; Music Recording Studio</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Where music finds its rhythm! Share your jamming &amp; recording experience on Google.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>https://www.google.com/maps/place/Naad+Jamroom+and+studio/@18.5607059,73.9393504,892m/data=!3m1!1e3!4m18!1m9!3m8!1s0x3bc2c366206c8fab:0x65510dbddf17da00!2sNaad+Jamroom+and+studio!8m2!3d18.5607008!4d73.9419307!9m1!1b1!16s%2Fg%2F11qgyk6z4x!3m7!1s0x3bc2c366206c8fab:0x65510dbddf17da00!8m2!3d18.5607008!4d73.9419307!9m1!1b1!16s%2Fg%2F11qgyk6z4x?entry=ttu&amp;g_ep=EgoyMDI2MTAyMC4wIKXMDSoASAFQAw%3D%3D</v>
+      </c>
+      <c r="G5" t="str">
+        <v>https://maps.app.goo.gl/ckY5Jtm92VDcsosd6</v>
+      </c>
+      <c r="H5" t="str">
+        <v>+91 73852 60556</v>
+      </c>
+      <c r="I5" t="str">
+        <v>917385260556</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>@naad_jamroom</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>Lane no 6, Parashar Housing Society, Pathare Thube Nagar Kharadi, Pune, Maharashtra 411014</v>
+      </c>
+      <c r="N5">
+        <v>4.9</v>
+      </c>
+      <c r="O5">
+        <v>125</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Band Jam Session; Audio Recording &amp; Tracking; Vocal Dubbing &amp; Booth; Mixing &amp; Mastering; Solo Instrument Practice; Podcast &amp; Voiceover</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Superb Acoustics &amp; Soundproofing; Top-Tier Drum Kit &amp; Tube Amps; Helpful &amp; Musician-Friendly Host; Cozy Mood Lighting &amp; Vibe; Crystal Clear Vocal Monitors; Affordable Hourly Jamming Rates; Clean &amp; Fully Air-Conditioned</v>
+      </c>
+      <c r="R5" t="str">
+        <v>/assets/naad-logo.png</v>
+      </c>
+      <c r="S5" t="str">
+        <v>#143736</v>
+      </c>
+      <c r="T5" t="str">
+        <v>#E89C3B</v>
+      </c>
+      <c r="U5" t="str">
+        <v>Active</v>
+      </c>
+      <c r="V5" t="str">
+        <v>/r/naadjamroom</v>
+      </c>
+      <c r="W5" t="str">
+        <v>/qr/naadjamroom</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>